<commit_message>
feat: add lesson for adding names and colors to new workbook
</commit_message>
<xml_diff>
--- a/colors.xlsx
+++ b/colors.xlsx
@@ -413,9 +413,70 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Names</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Colors</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dan</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Neal</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sara</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add lesson for using Excel formulas with Python
</commit_message>
<xml_diff>
--- a/colors.xlsx
+++ b/colors.xlsx
@@ -413,8 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -427,6 +432,11 @@
           <t>Colors</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Favorite Numbers</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -439,6 +449,9 @@
           <t>Blue</t>
         </is>
       </c>
+      <c r="C2" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -451,6 +464,9 @@
           <t>Purple</t>
         </is>
       </c>
+      <c r="C3" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -463,6 +479,9 @@
           <t>Green</t>
         </is>
       </c>
+      <c r="C4" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -474,6 +493,15 @@
         <is>
           <t>White</t>
         </is>
+      </c>
+      <c r="C5" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6">
+        <f>SUM(C2:C5)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>